<commit_message>
Mola na GC: os 40° passam a ser medidos a partir da chapa (até 50° da vertical)
Parâmetro renomeado para gc_angulo_minimo_base_graus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPzMHfEyU6XVTjYjHZdDvw
</commit_message>
<xml_diff>
--- a/data/parametros.xlsx
+++ b/data/parametros.xlsx
@@ -328,10 +328,10 @@
     <t>Passo do ângulo das barras inclinadas nos planos X, Y e Z (0 = só eixos). Barras entre duas esferas existentes ignoram o passo</t>
   </si>
   <si>
-    <t>gc_inclinacao_max_graus</t>
-  </si>
-  <si>
-    <t>Inclinação máxima de uma mola presa na GC, medida a partir da vertical (o aparato rígido em volta da esfera da GC limita)</t>
+    <t>gc_angulo_minimo_base_graus</t>
+  </si>
+  <si>
+    <t>Menor ângulo entre uma mola presa na GC e a chapa (base): 40° → a mola inclina no máximo 50° a partir da vertical (o aparato rígido em volta da esfera da GC limita)</t>
   </si>
   <si>
     <t>Código</t>

</xml_diff>

<commit_message>
Mola na GC: 40° medidos a partir da chapa (até 50° da vertical)
Parâmetro renomeado para gc_angulo_minimo_base_graus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPzMHfEyU6XVTjYjHZdDvw
</commit_message>
<xml_diff>
--- a/data/parametros.xlsx
+++ b/data/parametros.xlsx
@@ -328,10 +328,10 @@
     <t>Passo do ângulo das barras inclinadas nos planos X, Y e Z (0 = só eixos). Barras entre duas esferas existentes ignoram o passo</t>
   </si>
   <si>
-    <t>gc_inclinacao_max_graus</t>
-  </si>
-  <si>
-    <t>Inclinação máxima de uma mola presa na GC, medida a partir da vertical (o aparato rígido em volta da esfera da GC limita)</t>
+    <t>gc_angulo_minimo_base_graus</t>
+  </si>
+  <si>
+    <t>Menor ângulo entre uma mola presa na GC e a chapa (base): 40° → a mola inclina no máximo 50° a partir da vertical (o aparato rígido em volta da esfera da GC limita)</t>
   </si>
   <si>
     <t>Código</t>

</xml_diff>

<commit_message>
1.18: Kit 3 — cabo em dois cliques (ligações e clipes automáticos, bolinhas, plano de corte) e enrijecedor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPzMHfEyU6XVTjYjHZdDvw
</commit_message>
<xml_diff>
--- a/data/parametros.xlsx
+++ b/data/parametros.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="222">
   <si>
     <t>siMOLAdor: parâmetros (fonte dos dados do programa)</t>
   </si>
@@ -82,7 +82,7 @@
     <t>Placa: lado = vão × modulo_mm − placa_desconto_mm (nas duas direções).</t>
   </si>
   <si>
-    <t>Chapa de base: chapa_modulos_x × modulo_mm por chapa_modulos_y × modulo_mm.</t>
+    <t>Chapa de base: chapa_modulos_x × modulo_mm por chapa_modulos_y × modulo_mm. Cabo (Kit 3): cada pedaço sai da distância entre as esferas, em bolinhas (cabo_passo_mm).</t>
   </si>
   <si>
     <t>As colunas cinza (prévia) mostram o resultado com fórmulas só para conferência. Quem manda é o script.</t>
@@ -94,7 +94,7 @@
     <t>Amarelo = editar. Cinza-azulado = prévia calculada (não editar). Status: desenho (pranchas 2022), calculado, estimado (chute para o programa funcionar), medido (paquímetro), a medir.</t>
   </si>
   <si>
-    <t>Não renomeie a coluna Parâmetro (Geral) nem os títulos das colunas: o script lê por esses nomes. Tipos válidos: node = esfera, support = ligação de base, connector = ligações, bar = barra, cable = diagonal, plate = placa, ground = chapa. Fonte das quantidades: molamodel.com/pages/compare-products (08/10/2026).</t>
+    <t>Não renomeie a coluna Parâmetro (Geral) nem os títulos das colunas: o script lê por esses nomes. Tipos válidos: node = esfera, support = ligação de base, connector = ligações, bar = barra, cable = diagonal, plate = placa, ground = chapa, rope = cabo (Kit 3), accessory = ligações, clipes e anéis de cabo (entram sozinhos), stiffener = enrijecedor. Fonte das quantidades: molamodel.com/pages/compare-products (08/10/2026).</t>
   </si>
   <si>
     <t>Exemplo: medir a B6 e achar 75,2 mm → aba Peças, linha B6, coluna 'Comprimento medido' = 75,2 e Status = medido. As outras barras continuam pela regra.</t>
@@ -334,6 +334,69 @@
     <t>Menor ângulo entre uma mola presa na GC e a chapa (base): 40° → a mola inclina no máximo 50° a partir da vertical (o aparato rígido em volta da esfera da GC limita)</t>
   </si>
   <si>
+    <t>Cabos e enrijecedores (Kit 3)</t>
+  </si>
+  <si>
+    <t>cabo_passo_mm</t>
+  </si>
+  <si>
+    <t>Distância entre os centros de duas bolinhas vizinhas do cabo (corrente de bolinhas). Para medir: conte as bolinhas em 10 cm (≈ 31) e divida 100 mm pela contagem</t>
+  </si>
+  <si>
+    <t>fotos do Kit 3 (estimado)</t>
+  </si>
+  <si>
+    <t>cabo_bolinha_mm</t>
+  </si>
+  <si>
+    <t>Diâmetro da bolinha do cabo</t>
+  </si>
+  <si>
+    <t>cabo_rolo_mm</t>
+  </si>
+  <si>
+    <t>Comprimento do cabo que vem no Kit 3 (cortado na hora de montar)</t>
+  </si>
+  <si>
+    <t>site oficial</t>
+  </si>
+  <si>
+    <t>cabo_ligacao_mm</t>
+  </si>
+  <si>
+    <t>Ligação de cabo (CABLE C): da superfície da esfera até a ponta do anel (mola com ímã + anel)</t>
+  </si>
+  <si>
+    <t>cabo_clip_mm</t>
+  </si>
+  <si>
+    <t>Clip de cabo (CABLE CLIP C): do anel da CABLE C até o centro da bolinha da ponta do cabo</t>
+  </si>
+  <si>
+    <t>cabo_ajuste_mm</t>
+  </si>
+  <si>
+    <t>Quanto a CABLE C estica girando (esticador): absorve a sobra de menos de uma bolinha</t>
+  </si>
+  <si>
+    <t>manual do Kit 3 (estimado)</t>
+  </si>
+  <si>
+    <t>cabo_angulo_minimo_graus</t>
+  </si>
+  <si>
+    <t>Menor ângulo entre o cabo e outra peça na mesma esfera (a CABLE C precisa de lugar na esfera)</t>
+  </si>
+  <si>
+    <t>a confirmar</t>
+  </si>
+  <si>
+    <t>enrijecedor_diametro_mm</t>
+  </si>
+  <si>
+    <t>Diâmetro externo do enrijecedor (tubo transparente em volta da mola)</t>
+  </si>
+  <si>
     <t>Código</t>
   </si>
   <si>
@@ -511,6 +574,90 @@
     <t>Tamanho pela grade em Geral</t>
   </si>
   <si>
+    <t>CABLE</t>
+  </si>
+  <si>
+    <t>Cabo</t>
+  </si>
+  <si>
+    <t>rope</t>
+  </si>
+  <si>
+    <t>Corrente de bolinhas; vem um rolo de 3,35 m por Kit 3 e é cortado na montagem. Comprimento contado em bolinhas (régua do manual)</t>
+  </si>
+  <si>
+    <t>CABLE-C</t>
+  </si>
+  <si>
+    <t>Ligação de cabo (CABLE C)</t>
+  </si>
+  <si>
+    <t>accessory</t>
+  </si>
+  <si>
+    <t>esticador</t>
+  </si>
+  <si>
+    <t>Duas partes enroscadas: ímã na esfera, anel na outra ponta; girar ajusta o comprimento. Entra sozinha: 2 por cabo</t>
+  </si>
+  <si>
+    <t>CLIP-C</t>
+  </si>
+  <si>
+    <t>Clip de cabo (CABLE CLIP C)</t>
+  </si>
+  <si>
+    <t>Bolinha da ponta do cabo numa ponta, anel na outra; também une dois cabos. Entra sozinho: 2 por cabo</t>
+  </si>
+  <si>
+    <t>MCLIP-C</t>
+  </si>
+  <si>
+    <t>Clip de múltiplos cabos (M CABLE CLIP C)</t>
+  </si>
+  <si>
+    <t>Até 5 cabos numa só CABLE C. Ainda não usado pelo programa</t>
+  </si>
+  <si>
+    <t>RING-P</t>
+  </si>
+  <si>
+    <t>Anel de cabo pequeno (CABLE R)</t>
+  </si>
+  <si>
+    <t>Liga vários cabos num ponto (radial). Ainda não usado pelo programa</t>
+  </si>
+  <si>
+    <t>RING-M</t>
+  </si>
+  <si>
+    <t>Anel de cabo médio (CABLE R)</t>
+  </si>
+  <si>
+    <t>BS6</t>
+  </si>
+  <si>
+    <t>Enrijecedor B6 (BAR STIFFENER)</t>
+  </si>
+  <si>
+    <t>stiffener</t>
+  </si>
+  <si>
+    <t>deixa a mola rígida</t>
+  </si>
+  <si>
+    <t>Tubo transparente em volta da mola B6</t>
+  </si>
+  <si>
+    <t>BS12</t>
+  </si>
+  <si>
+    <t>Enrijecedor B12 (BAR STIFFENER)</t>
+  </si>
+  <si>
+    <t>Tubo transparente em volta da mola B12</t>
+  </si>
+  <si>
     <t>Kit</t>
   </si>
   <si>
@@ -538,7 +685,16 @@
     <t>Vermelho</t>
   </si>
   <si>
-    <t>Para incluir o Kit 3 ou 4: adicione uma linha aqui e uma coluna 'Kit 3' na aba Estoque.</t>
+    <t>Mola Structural Kit 3</t>
+  </si>
+  <si>
+    <t>#2F6FD6</t>
+  </si>
+  <si>
+    <t>Azul. Cabos (3,35 m), ligações e clipes de cabo, anéis, enrijecedores, B6, B12, D6x6, D6x12, RC90, 2 chapas</t>
+  </si>
+  <si>
+    <t>Para incluir o Kit 4 ou o Kit A: adicione uma linha aqui e uma coluna 'Kit N' na aba Estoque.</t>
   </si>
   <si>
     <t>Kit 1</t>
@@ -547,10 +703,13 @@
     <t>Kit 2</t>
   </si>
   <si>
+    <t>Kit 3</t>
+  </si>
+  <si>
     <t>Total</t>
   </si>
   <si>
-    <t>Conferir: Kit 1 = 122, Kit 2 = 145 (site oficial). A linha Total não é lida pelo script.</t>
+    <t>Conferir: Kit 1 = 122, Kit 2 = 145, Kit 3 = 205 (site oficial; o cabo conta como 1 peça). A linha Total não é lida pelo script.</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1195,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
@@ -1619,6 +1778,174 @@
       </c>
       <c r="F32" s="11" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B34" s="10">
+        <v>3.2</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="10">
+        <v>2.4</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" s="10">
+        <v>3350</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B37" s="10">
+        <v>16</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="10">
+        <v>9</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B39" s="10">
+        <v>4</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" s="10">
+        <v>20</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E40" s="9"/>
+      <c r="F40" s="11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B41" s="10">
+        <v>9</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1658,7 +1985,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1675,54 +2002,54 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>23</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
@@ -1740,18 +2067,18 @@
         <v>29</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -1769,18 +2096,18 @@
         <v>29</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" ht="35.05" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -1798,18 +2125,18 @@
         <v>29</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" ht="46.25" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="11"/>
@@ -1824,21 +2151,21 @@
       <c r="J5" s="10"/>
       <c r="K5" s="11"/>
       <c r="L5" s="11" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" ht="57.45" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -1853,21 +2180,21 @@
       <c r="J6" s="10"/>
       <c r="K6" s="11"/>
       <c r="L6" s="11" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D7" s="11">
         <v>4</v>
@@ -1883,22 +2210,22 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="11" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="M7" s="11"/>
     </row>
     <row r="8" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D8" s="11">
         <v>6</v>
@@ -1914,24 +2241,24 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="11" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>71</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D9" s="11">
         <v>12</v>
@@ -1947,7 +2274,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="11" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="L9" s="11" t="s">
         <v>29</v>
@@ -1956,13 +2283,13 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="D10" s="11">
         <v>4</v>
@@ -1980,22 +2307,22 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="11" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="M10" s="11"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="D11" s="11">
         <v>6</v>
@@ -2013,7 +2340,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
       <c r="K11" s="11" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="L11" s="11" t="s">
         <v>29</v>
@@ -2022,13 +2349,13 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="D12" s="11">
         <v>6</v>
@@ -2046,22 +2373,22 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="11" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="M12" s="11"/>
     </row>
     <row r="13" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="D13" s="11">
         <v>6</v>
@@ -2083,18 +2410,18 @@
         <v>29</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="D14" s="11">
         <v>12</v>
@@ -2116,18 +2443,18 @@
         <v>29</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
@@ -2145,7 +2472,241 @@
         <v>29</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>154</v>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12">
+        <f>cabo_rolo_mm</f>
+      </c>
+      <c r="G16" s="12">
+        <f>cabo_bolinha_mm</f>
+      </c>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12">
+        <f>cabo_ligacao_mm</f>
+      </c>
+      <c r="G17" s="12"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12">
+        <f>cabo_clip_mm</f>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="10">
+        <v>11</v>
+      </c>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="10">
+        <v>10</v>
+      </c>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="10">
+        <v>15</v>
+      </c>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M21" s="11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="D22" s="11">
+        <v>6</v>
+      </c>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12">
+        <f>IF(H22&lt;&gt;"",H22,D22*modulo_mm-barra_desconto_mm)</f>
+      </c>
+      <c r="G22" s="12">
+        <f>enrijecedor_diametro_mm</f>
+      </c>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="L22" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M22" s="11" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="D23" s="11">
+        <v>12</v>
+      </c>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12">
+        <f>IF(H23&lt;&gt;"",H23,D23*modulo_mm-barra_desconto_mm)</f>
+      </c>
+      <c r="G23" s="12">
+        <f>enrijecedor_diametro_mm</f>
+      </c>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M23" s="11" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2189,19 +2750,19 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>156</v>
+        <v>205</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>157</v>
+        <v>206</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2209,16 +2770,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>158</v>
+        <v>207</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>159</v>
+        <v>208</v>
       </c>
       <c r="D2" s="13">
         <v>122</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>160</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2226,21 +2787,38 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>162</v>
+        <v>211</v>
       </c>
       <c r="D3" s="13">
         <v>145</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>163</v>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="13">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D4" s="13">
+        <v>205</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>164</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2254,27 +2832,30 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
     <col min="2" max="3" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>165</v>
+        <v>217</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="B2" s="13">
         <v>12</v>
@@ -2282,10 +2863,13 @@
       <c r="C2" s="13">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="13">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B3" s="13">
         <v>4</v>
@@ -2293,10 +2877,13 @@
       <c r="C3" s="13">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D3" s="13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="B4" s="13">
         <v>48</v>
@@ -2304,10 +2891,13 @@
       <c r="C4" s="13">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D4" s="13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="B5" s="13">
         <v>0</v>
@@ -2315,10 +2905,13 @@
       <c r="C5" s="13">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D5" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B6" s="13">
         <v>0</v>
@@ -2326,10 +2919,13 @@
       <c r="C6" s="13">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D6" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="B7" s="13">
         <v>0</v>
@@ -2337,10 +2933,13 @@
       <c r="C7" s="13">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B8" s="13">
         <v>24</v>
@@ -2348,10 +2947,13 @@
       <c r="C8" s="13">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B9" s="13">
         <v>6</v>
@@ -2359,10 +2961,13 @@
       <c r="C9" s="13">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="B10" s="13">
         <v>0</v>
@@ -2370,10 +2975,13 @@
       <c r="C10" s="13">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D10" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="B11" s="13">
         <v>12</v>
@@ -2381,10 +2989,13 @@
       <c r="C11" s="13">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="B12" s="13">
         <v>12</v>
@@ -2392,10 +3003,13 @@
       <c r="C12" s="13">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D12" s="13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="B13" s="13">
         <v>0</v>
@@ -2403,10 +3017,13 @@
       <c r="C13" s="13">
         <v>3</v>
       </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D13" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="B14" s="13">
         <v>3</v>
@@ -2414,10 +3031,13 @@
       <c r="C14" s="13">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D14" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="B15" s="13">
         <v>1</v>
@@ -2425,21 +3045,139 @@
       <c r="C15" s="13">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>167</v>
-      </c>
-      <c r="B16" s="17">
-        <f>SUM(B2:B15)</f>
-      </c>
-      <c r="C16" s="17">
-        <f>SUM(C2:C15)</f>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>168</v>
+      <c r="D15" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="13">
+        <v>0</v>
+      </c>
+      <c r="C16" s="13">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="13">
+        <v>0</v>
+      </c>
+      <c r="C17" s="13">
+        <v>0</v>
+      </c>
+      <c r="D17" s="13">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="13">
+        <v>0</v>
+      </c>
+      <c r="C18" s="13">
+        <v>0</v>
+      </c>
+      <c r="D18" s="13">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="13">
+        <v>0</v>
+      </c>
+      <c r="C19" s="13">
+        <v>0</v>
+      </c>
+      <c r="D19" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B20" s="13">
+        <v>0</v>
+      </c>
+      <c r="C20" s="13">
+        <v>0</v>
+      </c>
+      <c r="D20" s="13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="B21" s="13">
+        <v>0</v>
+      </c>
+      <c r="C21" s="13">
+        <v>0</v>
+      </c>
+      <c r="D21" s="13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" s="13">
+        <v>0</v>
+      </c>
+      <c r="C22" s="13">
+        <v>0</v>
+      </c>
+      <c r="D22" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="13">
+        <v>0</v>
+      </c>
+      <c r="C23" s="13">
+        <v>0</v>
+      </c>
+      <c r="D23" s="13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="B24" s="17">
+        <f>SUM(B2:B23)</f>
+      </c>
+      <c r="C24" s="17">
+        <f>SUM(C2:C23)</f>
+      </c>
+      <c r="D24" s="17">
+        <f>SUM(D2:D23)</f>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1.5.0: Kit 3 — cabo em dois cliques (ligações e clipes automáticos, contado em bolinhas, plano de corte) e enrijecedor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPzMHfEyU6XVTjYjHZdDvw
</commit_message>
<xml_diff>
--- a/data/parametros.xlsx
+++ b/data/parametros.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="222">
   <si>
     <t>siMOLAdor: parâmetros (fonte dos dados do programa)</t>
   </si>
@@ -82,7 +82,7 @@
     <t>Placa: lado = vão × modulo_mm − placa_desconto_mm (nas duas direções).</t>
   </si>
   <si>
-    <t>Chapa de base: chapa_modulos_x × modulo_mm por chapa_modulos_y × modulo_mm.</t>
+    <t>Chapa de base: chapa_modulos_x × modulo_mm por chapa_modulos_y × modulo_mm. Cabo (Kit 3): cada pedaço sai da distância entre as esferas, em bolinhas (cabo_passo_mm).</t>
   </si>
   <si>
     <t>As colunas cinza (prévia) mostram o resultado com fórmulas só para conferência. Quem manda é o script.</t>
@@ -94,7 +94,7 @@
     <t>Amarelo = editar. Cinza-azulado = prévia calculada (não editar). Status: desenho (pranchas 2022), calculado, estimado (chute para o programa funcionar), medido (paquímetro), a medir.</t>
   </si>
   <si>
-    <t>Não renomeie a coluna Parâmetro (Geral) nem os títulos das colunas: o script lê por esses nomes. Tipos válidos: node = esfera, support = ligação de base, connector = ligações, bar = barra, cable = diagonal, plate = placa, ground = chapa. Fonte das quantidades: molamodel.com/pages/compare-products (08/10/2026).</t>
+    <t>Não renomeie a coluna Parâmetro (Geral) nem os títulos das colunas: o script lê por esses nomes. Tipos válidos: node = esfera, support = ligação de base, connector = ligações, bar = barra, cable = diagonal, plate = placa, ground = chapa, rope = cabo (Kit 3), accessory = ligações, clipes e anéis de cabo (entram sozinhos), stiffener = enrijecedor. Fonte das quantidades: molamodel.com/pages/compare-products (08/10/2026).</t>
   </si>
   <si>
     <t>Exemplo: medir a B6 e achar 75,2 mm → aba Peças, linha B6, coluna 'Comprimento medido' = 75,2 e Status = medido. As outras barras continuam pela regra.</t>
@@ -334,6 +334,69 @@
     <t>Menor ângulo entre uma mola presa na GC e a chapa (base): 40° → a mola inclina no máximo 50° a partir da vertical (o aparato rígido em volta da esfera da GC limita)</t>
   </si>
   <si>
+    <t>Cabos e enrijecedores (Kit 3)</t>
+  </si>
+  <si>
+    <t>cabo_passo_mm</t>
+  </si>
+  <si>
+    <t>Distância entre os centros de duas bolinhas vizinhas do cabo (corrente de bolinhas). Para medir: conte as bolinhas em 10 cm (≈ 31) e divida 100 mm pela contagem</t>
+  </si>
+  <si>
+    <t>fotos do Kit 3 (estimado)</t>
+  </si>
+  <si>
+    <t>cabo_bolinha_mm</t>
+  </si>
+  <si>
+    <t>Diâmetro da bolinha do cabo</t>
+  </si>
+  <si>
+    <t>cabo_rolo_mm</t>
+  </si>
+  <si>
+    <t>Comprimento do cabo que vem no Kit 3 (cortado na hora de montar)</t>
+  </si>
+  <si>
+    <t>site oficial</t>
+  </si>
+  <si>
+    <t>cabo_ligacao_mm</t>
+  </si>
+  <si>
+    <t>Ligação de cabo (CABLE C): da superfície da esfera até a ponta do anel (mola com ímã + anel)</t>
+  </si>
+  <si>
+    <t>cabo_clip_mm</t>
+  </si>
+  <si>
+    <t>Clip de cabo (CABLE CLIP C): do anel da CABLE C até o centro da bolinha da ponta do cabo</t>
+  </si>
+  <si>
+    <t>cabo_ajuste_mm</t>
+  </si>
+  <si>
+    <t>Quanto a CABLE C estica girando (esticador): absorve a sobra de menos de uma bolinha</t>
+  </si>
+  <si>
+    <t>manual do Kit 3 (estimado)</t>
+  </si>
+  <si>
+    <t>cabo_angulo_minimo_graus</t>
+  </si>
+  <si>
+    <t>Menor ângulo entre o cabo e outra peça na mesma esfera (a CABLE C precisa de lugar na esfera)</t>
+  </si>
+  <si>
+    <t>a confirmar</t>
+  </si>
+  <si>
+    <t>enrijecedor_diametro_mm</t>
+  </si>
+  <si>
+    <t>Diâmetro externo do enrijecedor (tubo transparente em volta da mola)</t>
+  </si>
+  <si>
     <t>Código</t>
   </si>
   <si>
@@ -511,6 +574,90 @@
     <t>Tamanho pela grade em Geral</t>
   </si>
   <si>
+    <t>CABLE</t>
+  </si>
+  <si>
+    <t>Cabo</t>
+  </si>
+  <si>
+    <t>rope</t>
+  </si>
+  <si>
+    <t>Corrente de bolinhas; vem um rolo de 3,35 m por Kit 3 e é cortado na montagem. Comprimento contado em bolinhas (régua do manual)</t>
+  </si>
+  <si>
+    <t>CABLE-C</t>
+  </si>
+  <si>
+    <t>Ligação de cabo (CABLE C)</t>
+  </si>
+  <si>
+    <t>accessory</t>
+  </si>
+  <si>
+    <t>esticador</t>
+  </si>
+  <si>
+    <t>Duas partes enroscadas: ímã na esfera, anel na outra ponta; girar ajusta o comprimento. Entra sozinha: 2 por cabo</t>
+  </si>
+  <si>
+    <t>CLIP-C</t>
+  </si>
+  <si>
+    <t>Clip de cabo (CABLE CLIP C)</t>
+  </si>
+  <si>
+    <t>Bolinha da ponta do cabo numa ponta, anel na outra; também une dois cabos. Entra sozinho: 2 por cabo</t>
+  </si>
+  <si>
+    <t>MCLIP-C</t>
+  </si>
+  <si>
+    <t>Clip de múltiplos cabos (M CABLE CLIP C)</t>
+  </si>
+  <si>
+    <t>Até 5 cabos numa só CABLE C. Ainda não usado pelo programa</t>
+  </si>
+  <si>
+    <t>RING-P</t>
+  </si>
+  <si>
+    <t>Anel de cabo pequeno (CABLE R)</t>
+  </si>
+  <si>
+    <t>Liga vários cabos num ponto (radial). Ainda não usado pelo programa</t>
+  </si>
+  <si>
+    <t>RING-M</t>
+  </si>
+  <si>
+    <t>Anel de cabo médio (CABLE R)</t>
+  </si>
+  <si>
+    <t>BS6</t>
+  </si>
+  <si>
+    <t>Enrijecedor B6 (BAR STIFFENER)</t>
+  </si>
+  <si>
+    <t>stiffener</t>
+  </si>
+  <si>
+    <t>deixa a mola rígida</t>
+  </si>
+  <si>
+    <t>Tubo transparente em volta da mola B6</t>
+  </si>
+  <si>
+    <t>BS12</t>
+  </si>
+  <si>
+    <t>Enrijecedor B12 (BAR STIFFENER)</t>
+  </si>
+  <si>
+    <t>Tubo transparente em volta da mola B12</t>
+  </si>
+  <si>
     <t>Kit</t>
   </si>
   <si>
@@ -538,7 +685,16 @@
     <t>Vermelho</t>
   </si>
   <si>
-    <t>Para incluir o Kit 3 ou 4: adicione uma linha aqui e uma coluna 'Kit 3' na aba Estoque.</t>
+    <t>Mola Structural Kit 3</t>
+  </si>
+  <si>
+    <t>#2F6FD6</t>
+  </si>
+  <si>
+    <t>Azul. Cabos (3,35 m), ligações e clipes de cabo, anéis, enrijecedores, B6, B12, D6x6, D6x12, RC90, 2 chapas</t>
+  </si>
+  <si>
+    <t>Para incluir o Kit 4 ou o Kit A: adicione uma linha aqui e uma coluna 'Kit N' na aba Estoque.</t>
   </si>
   <si>
     <t>Kit 1</t>
@@ -547,10 +703,13 @@
     <t>Kit 2</t>
   </si>
   <si>
+    <t>Kit 3</t>
+  </si>
+  <si>
     <t>Total</t>
   </si>
   <si>
-    <t>Conferir: Kit 1 = 122, Kit 2 = 145 (site oficial). A linha Total não é lida pelo script.</t>
+    <t>Conferir: Kit 1 = 122, Kit 2 = 145, Kit 3 = 205 (site oficial; o cabo conta como 1 peça). A linha Total não é lida pelo script.</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1195,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
@@ -1619,6 +1778,174 @@
       </c>
       <c r="F32" s="11" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B34" s="10">
+        <v>3.2</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="10">
+        <v>2.4</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" s="10">
+        <v>3350</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B37" s="10">
+        <v>16</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="10">
+        <v>9</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B39" s="10">
+        <v>4</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" s="10">
+        <v>20</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E40" s="9"/>
+      <c r="F40" s="11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B41" s="10">
+        <v>9</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1658,7 +1985,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1675,54 +2002,54 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>23</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
@@ -1740,18 +2067,18 @@
         <v>29</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -1769,18 +2096,18 @@
         <v>29</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" ht="35.05" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -1798,18 +2125,18 @@
         <v>29</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" ht="46.25" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="11"/>
@@ -1824,21 +2151,21 @@
       <c r="J5" s="10"/>
       <c r="K5" s="11"/>
       <c r="L5" s="11" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" ht="57.45" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -1853,21 +2180,21 @@
       <c r="J6" s="10"/>
       <c r="K6" s="11"/>
       <c r="L6" s="11" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D7" s="11">
         <v>4</v>
@@ -1883,22 +2210,22 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="11" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="M7" s="11"/>
     </row>
     <row r="8" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D8" s="11">
         <v>6</v>
@@ -1914,24 +2241,24 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="11" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>71</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="D9" s="11">
         <v>12</v>
@@ -1947,7 +2274,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="11" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="L9" s="11" t="s">
         <v>29</v>
@@ -1956,13 +2283,13 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="D10" s="11">
         <v>4</v>
@@ -1980,22 +2307,22 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="11" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="M10" s="11"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="D11" s="11">
         <v>6</v>
@@ -2013,7 +2340,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
       <c r="K11" s="11" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="L11" s="11" t="s">
         <v>29</v>
@@ -2022,13 +2349,13 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="D12" s="11">
         <v>6</v>
@@ -2046,22 +2373,22 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="11" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="M12" s="11"/>
     </row>
     <row r="13" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="D13" s="11">
         <v>6</v>
@@ -2083,18 +2410,18 @@
         <v>29</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="D14" s="11">
         <v>12</v>
@@ -2116,18 +2443,18 @@
         <v>29</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
@@ -2145,7 +2472,241 @@
         <v>29</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>154</v>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12">
+        <f>cabo_rolo_mm</f>
+      </c>
+      <c r="G16" s="12">
+        <f>cabo_bolinha_mm</f>
+      </c>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12">
+        <f>cabo_ligacao_mm</f>
+      </c>
+      <c r="G17" s="12"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12">
+        <f>cabo_clip_mm</f>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="10">
+        <v>11</v>
+      </c>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="10">
+        <v>10</v>
+      </c>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="10">
+        <v>15</v>
+      </c>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M21" s="11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="D22" s="11">
+        <v>6</v>
+      </c>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12">
+        <f>IF(H22&lt;&gt;"",H22,D22*modulo_mm-barra_desconto_mm)</f>
+      </c>
+      <c r="G22" s="12">
+        <f>enrijecedor_diametro_mm</f>
+      </c>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="L22" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M22" s="11" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="D23" s="11">
+        <v>12</v>
+      </c>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12">
+        <f>IF(H23&lt;&gt;"",H23,D23*modulo_mm-barra_desconto_mm)</f>
+      </c>
+      <c r="G23" s="12">
+        <f>enrijecedor_diametro_mm</f>
+      </c>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M23" s="11" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -2189,19 +2750,19 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>156</v>
+        <v>205</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>157</v>
+        <v>206</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2209,16 +2770,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>158</v>
+        <v>207</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>159</v>
+        <v>208</v>
       </c>
       <c r="D2" s="13">
         <v>122</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>160</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2226,21 +2787,38 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>162</v>
+        <v>211</v>
       </c>
       <c r="D3" s="13">
         <v>145</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>163</v>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="13">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D4" s="13">
+        <v>205</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>164</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2254,27 +2832,30 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
     <col min="2" max="3" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>165</v>
+        <v>217</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="B2" s="13">
         <v>12</v>
@@ -2282,10 +2863,13 @@
       <c r="C2" s="13">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="13">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B3" s="13">
         <v>4</v>
@@ -2293,10 +2877,13 @@
       <c r="C3" s="13">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D3" s="13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="B4" s="13">
         <v>48</v>
@@ -2304,10 +2891,13 @@
       <c r="C4" s="13">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D4" s="13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="B5" s="13">
         <v>0</v>
@@ -2315,10 +2905,13 @@
       <c r="C5" s="13">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D5" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B6" s="13">
         <v>0</v>
@@ -2326,10 +2919,13 @@
       <c r="C6" s="13">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D6" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="B7" s="13">
         <v>0</v>
@@ -2337,10 +2933,13 @@
       <c r="C7" s="13">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B8" s="13">
         <v>24</v>
@@ -2348,10 +2947,13 @@
       <c r="C8" s="13">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D8" s="13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B9" s="13">
         <v>6</v>
@@ -2359,10 +2961,13 @@
       <c r="C9" s="13">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="B10" s="13">
         <v>0</v>
@@ -2370,10 +2975,13 @@
       <c r="C10" s="13">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D10" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="B11" s="13">
         <v>12</v>
@@ -2381,10 +2989,13 @@
       <c r="C11" s="13">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="B12" s="13">
         <v>12</v>
@@ -2392,10 +3003,13 @@
       <c r="C12" s="13">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D12" s="13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="B13" s="13">
         <v>0</v>
@@ -2403,10 +3017,13 @@
       <c r="C13" s="13">
         <v>3</v>
       </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D13" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="B14" s="13">
         <v>3</v>
@@ -2414,10 +3031,13 @@
       <c r="C14" s="13">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D14" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="B15" s="13">
         <v>1</v>
@@ -2425,21 +3045,139 @@
       <c r="C15" s="13">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>167</v>
-      </c>
-      <c r="B16" s="17">
-        <f>SUM(B2:B15)</f>
-      </c>
-      <c r="C16" s="17">
-        <f>SUM(C2:C15)</f>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>168</v>
+      <c r="D15" s="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="13">
+        <v>0</v>
+      </c>
+      <c r="C16" s="13">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="13">
+        <v>0</v>
+      </c>
+      <c r="C17" s="13">
+        <v>0</v>
+      </c>
+      <c r="D17" s="13">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B18" s="13">
+        <v>0</v>
+      </c>
+      <c r="C18" s="13">
+        <v>0</v>
+      </c>
+      <c r="D18" s="13">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="13">
+        <v>0</v>
+      </c>
+      <c r="C19" s="13">
+        <v>0</v>
+      </c>
+      <c r="D19" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B20" s="13">
+        <v>0</v>
+      </c>
+      <c r="C20" s="13">
+        <v>0</v>
+      </c>
+      <c r="D20" s="13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="B21" s="13">
+        <v>0</v>
+      </c>
+      <c r="C21" s="13">
+        <v>0</v>
+      </c>
+      <c r="D21" s="13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" s="13">
+        <v>0</v>
+      </c>
+      <c r="C22" s="13">
+        <v>0</v>
+      </c>
+      <c r="D22" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="13">
+        <v>0</v>
+      </c>
+      <c r="C23" s="13">
+        <v>0</v>
+      </c>
+      <c r="D23" s="13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="B24" s="17">
+        <f>SUM(B2:B23)</f>
+      </c>
+      <c r="C24" s="17">
+        <f>SUM(C2:C23)</f>
+      </c>
+      <c r="D24" s="17">
+        <f>SUM(D2:D23)</f>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cabo calibrado: diagonal de 12M × 12M com 60 bolinhas (passo 3,15 mm)
</commit_message>
<xml_diff>
--- a/data/parametros.xlsx
+++ b/data/parametros.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="224">
   <si>
     <t>siMOLAdor: parâmetros (fonte dos dados do programa)</t>
   </si>
@@ -343,13 +343,19 @@
     <t>Distância entre os centros de duas bolinhas vizinhas do cabo (corrente de bolinhas). Para medir: conte as bolinhas em 10 cm (≈ 31) e divida 100 mm pela contagem</t>
   </si>
   <si>
+    <t>calibrado pela equipe (26/10): a diagonal de um quadrado de 12M x 12M pede 60 bolinhas para ficar esticada</t>
+  </si>
+  <si>
+    <t>calibrado</t>
+  </si>
+  <si>
+    <t>cabo_bolinha_mm</t>
+  </si>
+  <si>
+    <t>Diâmetro da bolinha do cabo</t>
+  </si>
+  <si>
     <t>fotos do Kit 3 (estimado)</t>
-  </si>
-  <si>
-    <t>cabo_bolinha_mm</t>
-  </si>
-  <si>
-    <t>Diâmetro da bolinha do cabo</t>
   </si>
   <si>
     <t>cabo_rolo_mm</t>
@@ -1795,7 +1801,7 @@
         <v>97</v>
       </c>
       <c r="B34" s="10">
-        <v>3.2</v>
+        <v>3.15</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>26</v>
@@ -1807,12 +1813,12 @@
         <v>99</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>43</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B35" s="10">
         <v>2.4</v>
@@ -1821,10 +1827,10 @@
         <v>26</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F35" s="11" t="s">
         <v>43</v>
@@ -1832,7 +1838,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B36" s="10">
         <v>3350</v>
@@ -1841,10 +1847,10 @@
         <v>26</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F36" s="11" t="s">
         <v>71</v>
@@ -1852,7 +1858,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B37" s="10">
         <v>16</v>
@@ -1861,10 +1867,10 @@
         <v>26</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F37" s="11" t="s">
         <v>43</v>
@@ -1872,7 +1878,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B38" s="10">
         <v>9</v>
@@ -1881,10 +1887,10 @@
         <v>26</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F38" s="11" t="s">
         <v>43</v>
@@ -1892,7 +1898,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B39" s="10">
         <v>4</v>
@@ -1901,10 +1907,10 @@
         <v>26</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F39" s="11" t="s">
         <v>43</v>
@@ -1912,7 +1918,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B40" s="10">
         <v>20</v>
@@ -1921,16 +1927,16 @@
         <v>80</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E40" s="9"/>
       <c r="F40" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B41" s="10">
         <v>9</v>
@@ -1939,10 +1945,10 @@
         <v>26</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F41" s="11" t="s">
         <v>43</v>
@@ -2002,54 +2008,54 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>23</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
@@ -2067,18 +2073,18 @@
         <v>29</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -2096,18 +2102,18 @@
         <v>29</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" ht="35.05" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -2125,18 +2131,18 @@
         <v>29</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" ht="46.25" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>139</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="11"/>
@@ -2151,21 +2157,21 @@
       <c r="J5" s="10"/>
       <c r="K5" s="11"/>
       <c r="L5" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" ht="57.45" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -2180,21 +2186,21 @@
       <c r="J6" s="10"/>
       <c r="K6" s="11"/>
       <c r="L6" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D7" s="11">
         <v>4</v>
@@ -2210,22 +2216,22 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="11" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="M7" s="11"/>
     </row>
     <row r="8" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D8" s="11">
         <v>6</v>
@@ -2241,24 +2247,24 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="11" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>71</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D9" s="11">
         <v>12</v>
@@ -2274,7 +2280,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="11" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L9" s="11" t="s">
         <v>29</v>
@@ -2283,13 +2289,13 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D10" s="11">
         <v>4</v>
@@ -2307,22 +2313,22 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="M10" s="11"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>162</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>160</v>
       </c>
       <c r="D11" s="11">
         <v>6</v>
@@ -2340,7 +2346,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
       <c r="K11" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L11" s="11" t="s">
         <v>29</v>
@@ -2349,13 +2355,13 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D12" s="11">
         <v>6</v>
@@ -2373,22 +2379,22 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="M12" s="11"/>
     </row>
     <row r="13" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D13" s="11">
         <v>6</v>
@@ -2410,18 +2416,18 @@
         <v>29</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="D14" s="11">
         <v>12</v>
@@ -2443,18 +2449,18 @@
         <v>29</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
@@ -2472,18 +2478,18 @@
         <v>29</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
@@ -2497,24 +2503,24 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
       <c r="K16" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L16" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
@@ -2526,24 +2532,24 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
       <c r="K17" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="L17" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
@@ -2559,18 +2565,18 @@
         <v>43</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
@@ -2586,18 +2592,18 @@
         <v>43</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
@@ -2613,18 +2619,18 @@
         <v>43</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
@@ -2640,18 +2646,18 @@
         <v>43</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D22" s="11">
         <v>6</v>
@@ -2667,24 +2673,24 @@
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
       <c r="K22" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L22" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M22" s="11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D23" s="11">
         <v>12</v>
@@ -2700,13 +2706,13 @@
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
       <c r="K23" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L23" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M23" s="11" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2750,19 +2756,19 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2770,16 +2776,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D2" s="13">
         <v>122</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2787,16 +2793,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D3" s="13">
         <v>145</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2804,21 +2810,21 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D4" s="13">
         <v>205</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -2841,21 +2847,21 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B2" s="13">
         <v>12</v>
@@ -2869,7 +2875,7 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B3" s="13">
         <v>4</v>
@@ -2883,7 +2889,7 @@
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B4" s="13">
         <v>48</v>
@@ -2897,7 +2903,7 @@
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B5" s="13">
         <v>0</v>
@@ -2911,7 +2917,7 @@
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B6" s="13">
         <v>0</v>
@@ -2925,7 +2931,7 @@
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B7" s="13">
         <v>0</v>
@@ -2939,7 +2945,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B8" s="13">
         <v>24</v>
@@ -2953,7 +2959,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B9" s="13">
         <v>6</v>
@@ -2967,7 +2973,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B10" s="13">
         <v>0</v>
@@ -2981,7 +2987,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B11" s="13">
         <v>12</v>
@@ -2995,7 +3001,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B12" s="13">
         <v>12</v>
@@ -3009,7 +3015,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B13" s="13">
         <v>0</v>
@@ -3023,7 +3029,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B14" s="13">
         <v>3</v>
@@ -3037,7 +3043,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B15" s="13">
         <v>1</v>
@@ -3051,7 +3057,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B16" s="13">
         <v>0</v>
@@ -3065,7 +3071,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B17" s="13">
         <v>0</v>
@@ -3079,7 +3085,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B18" s="13">
         <v>0</v>
@@ -3093,7 +3099,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B19" s="13">
         <v>0</v>
@@ -3107,7 +3113,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B20" s="13">
         <v>0</v>
@@ -3121,7 +3127,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B21" s="13">
         <v>0</v>
@@ -3135,7 +3141,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B22" s="13">
         <v>0</v>
@@ -3149,7 +3155,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B23" s="13">
         <v>0</v>
@@ -3163,7 +3169,7 @@
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B24" s="17">
         <f>SUM(B2:B23)</f>
@@ -3177,7 +3183,7 @@
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cabo preso em cabo (pendurais): clip no meio do cabo, referências verde e amarela, ponto de cabo que desce bolinha a bolinha; copiar e colar cabos inteiros
</commit_message>
<xml_diff>
--- a/data/parametros.xlsx
+++ b/data/parametros.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="226">
   <si>
     <t>siMOLAdor: parâmetros (fonte dos dados do programa)</t>
   </si>
@@ -377,6 +377,12 @@
   </si>
   <si>
     <t>Clip de cabo (CABLE CLIP C): do anel da CABLE C até o centro da bolinha da ponta do cabo</t>
+  </si>
+  <si>
+    <t>cabo_pendural_mm</t>
+  </si>
+  <si>
+    <t>Cabo preso no meio de outro (pendural): do centro da bolinha do cabo principal, no furo do meio do CABLE CLIP C, ao centro da primeira bolinha do pendural</t>
   </si>
   <si>
     <t>cabo_ajuste_mm</t>
@@ -1201,7 +1207,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
@@ -1901,7 +1907,7 @@
         <v>111</v>
       </c>
       <c r="B39" s="10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>26</v>
@@ -1910,7 +1916,7 @@
         <v>112</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="F39" s="11" t="s">
         <v>43</v>
@@ -1918,39 +1924,59 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B40" s="10">
+        <v>4</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D40" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B40" s="10">
-        <v>20</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D40" s="9" t="s">
+      <c r="E40" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="E40" s="9"/>
       <c r="F40" s="11" t="s">
-        <v>116</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B41" s="10">
+        <v>20</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D41" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="B41" s="10">
+      <c r="E41" s="9"/>
+      <c r="F41" s="11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B42" s="10">
         <v>9</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C42" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D41" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="E41" s="9" t="s">
+      <c r="D42" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="E42" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F41" s="11" t="s">
+      <c r="F42" s="11" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2008,54 +2034,54 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>23</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
@@ -2073,18 +2099,18 @@
         <v>29</v>
       </c>
       <c r="M2" s="11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -2102,18 +2128,18 @@
         <v>29</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" ht="35.05" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -2131,18 +2157,18 @@
         <v>29</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" ht="46.25" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>143</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>141</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="11"/>
@@ -2157,21 +2183,21 @@
       <c r="J5" s="10"/>
       <c r="K5" s="11"/>
       <c r="L5" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" ht="57.45" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -2186,21 +2212,21 @@
       <c r="J6" s="10"/>
       <c r="K6" s="11"/>
       <c r="L6" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D7" s="11">
         <v>4</v>
@@ -2216,22 +2242,22 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="M7" s="11"/>
     </row>
     <row r="8" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D8" s="11">
         <v>6</v>
@@ -2247,24 +2273,24 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>71</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D9" s="11">
         <v>12</v>
@@ -2280,7 +2306,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L9" s="11" t="s">
         <v>29</v>
@@ -2289,13 +2315,13 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D10" s="11">
         <v>4</v>
@@ -2313,22 +2339,22 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="M10" s="11"/>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>162</v>
       </c>
       <c r="D11" s="11">
         <v>6</v>
@@ -2346,7 +2372,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
       <c r="K11" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L11" s="11" t="s">
         <v>29</v>
@@ -2355,13 +2381,13 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D12" s="11">
         <v>6</v>
@@ -2379,22 +2405,22 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="M12" s="11"/>
     </row>
     <row r="13" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D13" s="11">
         <v>6</v>
@@ -2416,18 +2442,18 @@
         <v>29</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>172</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="D14" s="11">
         <v>12</v>
@@ -2449,18 +2475,18 @@
         <v>29</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
@@ -2478,18 +2504,18 @@
         <v>29</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
@@ -2503,24 +2529,24 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
       <c r="K16" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L16" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
@@ -2532,24 +2558,24 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
       <c r="K17" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="L17" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
@@ -2565,18 +2591,18 @@
         <v>43</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
@@ -2592,18 +2618,18 @@
         <v>43</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
@@ -2619,18 +2645,18 @@
         <v>43</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
@@ -2646,18 +2672,18 @@
         <v>43</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D22" s="11">
         <v>6</v>
@@ -2673,24 +2699,24 @@
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
       <c r="K22" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="L22" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M22" s="11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D23" s="11">
         <v>12</v>
@@ -2706,13 +2732,13 @@
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
       <c r="K23" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="L23" s="11" t="s">
         <v>43</v>
       </c>
       <c r="M23" s="11" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -2756,19 +2782,19 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2776,16 +2802,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D2" s="13">
         <v>122</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2793,16 +2819,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D3" s="13">
         <v>145</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2810,21 +2836,21 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D4" s="13">
         <v>205</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -2847,21 +2873,21 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B2" s="13">
         <v>12</v>
@@ -2875,7 +2901,7 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B3" s="13">
         <v>4</v>
@@ -2889,7 +2915,7 @@
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B4" s="13">
         <v>48</v>
@@ -2903,7 +2929,7 @@
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B5" s="13">
         <v>0</v>
@@ -2917,7 +2943,7 @@
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B6" s="13">
         <v>0</v>
@@ -2931,7 +2957,7 @@
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B7" s="13">
         <v>0</v>
@@ -2945,7 +2971,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B8" s="13">
         <v>24</v>
@@ -2959,7 +2985,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B9" s="13">
         <v>6</v>
@@ -2973,7 +2999,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B10" s="13">
         <v>0</v>
@@ -2987,7 +3013,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B11" s="13">
         <v>12</v>
@@ -3001,7 +3027,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B12" s="13">
         <v>12</v>
@@ -3015,7 +3041,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B13" s="13">
         <v>0</v>
@@ -3029,7 +3055,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B14" s="13">
         <v>3</v>
@@ -3043,7 +3069,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B15" s="13">
         <v>1</v>
@@ -3057,7 +3083,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B16" s="13">
         <v>0</v>
@@ -3071,7 +3097,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B17" s="13">
         <v>0</v>
@@ -3085,7 +3111,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B18" s="13">
         <v>0</v>
@@ -3099,7 +3125,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B19" s="13">
         <v>0</v>
@@ -3113,7 +3139,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B20" s="13">
         <v>0</v>
@@ -3127,7 +3153,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B21" s="13">
         <v>0</v>
@@ -3141,7 +3167,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B22" s="13">
         <v>0</v>
@@ -3155,7 +3181,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B23" s="13">
         <v>0</v>
@@ -3169,7 +3195,7 @@
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B24" s="17">
         <f>SUM(B2:B23)</f>
@@ -3183,7 +3209,7 @@
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>